<commit_message>
feat: Importacion de productos via Excel y plantillas
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_productos.xlsx
+++ b/assets/templates/plantilla_productos.xlsx
@@ -1,26 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\CarePharm\dist\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B473712-9C7A-42C9-B30A-BF92BE50D9A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="LISTA EXCEL" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="LISTA EXCEL" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
   <si>
     <t>COD.DIGEMID</t>
   </si>
@@ -37,7 +28,10 @@
     <t>LABORATORIO</t>
   </si>
   <si>
-    <t>F.V.</t>
+    <t>F. VENCIMIENTO (dd/mm/aaaa)</t>
+  </si>
+  <si>
+    <t>F. FABRICACION (dd/mm/aaaa)</t>
   </si>
   <si>
     <t>CANT x CAJA</t>
@@ -82,7 +76,10 @@
     <t>F.COMPRA</t>
   </si>
   <si>
-    <t>REGISTRO SA.</t>
+    <t>PROD. CONTROLADO (SI/NO)</t>
+  </si>
+  <si>
+    <t>ANAQUEL</t>
   </si>
   <si>
     <t>cod_digemid</t>
@@ -100,6 +97,12 @@
     <t>laboratorio</t>
   </si>
   <si>
+    <t>reg_san</t>
+  </si>
+  <si>
+    <t>fecha_fabricacion</t>
+  </si>
+  <si>
     <t>fecha_venc</t>
   </si>
   <si>
@@ -145,10 +148,10 @@
     <t>fecha_compra</t>
   </si>
   <si>
-    <t>reg_san</t>
-  </si>
-  <si>
-    <t>1211041</t>
+    <t>is_controlled</t>
+  </si>
+  <si>
+    <t>anaquel</t>
   </si>
   <si>
     <t>BICARBONATO DE SODIO POTE X 500</t>
@@ -163,75 +166,60 @@
     <t>OLCASA S.A.C.</t>
   </si>
   <si>
-    <t>1/25/2026</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>35167</t>
-  </si>
-  <si>
-    <t>S/ 15.96</t>
-  </si>
-  <si>
-    <t>S/ 1.13</t>
+    <t>01/15/2024</t>
+  </si>
+  <si>
+    <t>01/25/2026</t>
   </si>
   <si>
     <t>F001-0000857</t>
   </si>
   <si>
-    <t>S/ 2.00</t>
-  </si>
-  <si>
-    <t>S/ 1.80</t>
-  </si>
-  <si>
-    <t>7.9641-15 F001-0000657</t>
-  </si>
-  <si>
-    <t>2300657+90</t>
+    <t>2.00</t>
+  </si>
+  <si>
+    <t>1.80</t>
   </si>
   <si>
     <t>IQUITOS</t>
   </si>
   <si>
-    <t>5/05/2026</t>
-  </si>
-  <si>
-    <t>123456</t>
+    <t>05/05/2026</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>A-1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="9"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
+      <i/>
+      <color rgb="FF666666"/>
+      <sz val="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="8"/>
-      <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -361,7 +349,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -371,44 +359,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -436,31 +424,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -488,23 +459,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -516,150 +470,208 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:U103"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X103"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -667,21 +679,26 @@
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="22" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="28" customWidth="1"/>
-    <col min="19" max="19" width="16" customWidth="1"/>
-    <col min="20" max="21" width="14" customWidth="1"/>
+    <col min="7" max="7" width="17.285714285714285" customWidth="1"/>
+    <col min="8" max="8" width="15.428571428571429" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="20" customWidth="1"/>
+    <col min="19" max="19" width="28" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="21" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="24" customWidth="1"/>
+    <col min="24" max="24" width="15" customWidth="1"/>
+    <col min="25" max="48" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="42" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -697,14 +714,14 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>20</v>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>7</v>
@@ -715,164 +732,191 @@
       <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="P1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" ht="12.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="T2" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="U2" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="12" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="V2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="W2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>1211041</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>60</v>
+        <v>50</v>
+      </c>
+      <c r="F3" s="8">
+        <v>123456</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="I3" s="8">
+        <v>1</v>
+      </c>
+      <c r="J3" s="8">
+        <v>12</v>
+      </c>
+      <c r="K3" s="8">
+        <v>35167</v>
+      </c>
+      <c r="L3" s="8">
+        <v>5.96</v>
+      </c>
+      <c r="M3" s="8">
+        <v>1.13</v>
+      </c>
+      <c r="N3" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="8" t="s">
+      <c r="O3" s="9"/>
+      <c r="P3" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="Q3" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="R3" s="8">
+        <v>2023145620123</v>
+      </c>
+      <c r="S3" s="8">
+        <v>23006570090</v>
+      </c>
+      <c r="T3" s="9"/>
+      <c r="U3" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="V3" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="S3" s="9"/>
-      <c r="T3" s="8" t="s">
+      <c r="W3" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="U3" s="8" t="s">
+      <c r="X3" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="4" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -894,8 +938,11 @@
       <c r="S4" s="9"/>
       <c r="T4" s="9"/>
       <c r="U4" s="9"/>
-    </row>
-    <row r="5" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V4" s="9"/>
+      <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -917,8 +964,11 @@
       <c r="S5" s="9"/>
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
-    </row>
-    <row r="6" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V5" s="9"/>
+      <c r="W5" s="9"/>
+      <c r="X5" s="9"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -940,8 +990,11 @@
       <c r="S6" s="9"/>
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
-    </row>
-    <row r="7" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V6" s="9"/>
+      <c r="W6" s="9"/>
+      <c r="X6" s="9"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -963,8 +1016,11 @@
       <c r="S7" s="9"/>
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
-    </row>
-    <row r="8" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V7" s="9"/>
+      <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -986,8 +1042,11 @@
       <c r="S8" s="9"/>
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
-    </row>
-    <row r="9" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V8" s="9"/>
+      <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -1009,8 +1068,11 @@
       <c r="S9" s="9"/>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
-    </row>
-    <row r="10" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V9" s="9"/>
+      <c r="W9" s="9"/>
+      <c r="X9" s="9"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -1032,8 +1094,11 @@
       <c r="S10" s="9"/>
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
-    </row>
-    <row r="11" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V10" s="9"/>
+      <c r="W10" s="9"/>
+      <c r="X10" s="9"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -1055,8 +1120,11 @@
       <c r="S11" s="9"/>
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
-    </row>
-    <row r="12" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V11" s="9"/>
+      <c r="W11" s="9"/>
+      <c r="X11" s="9"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1078,8 +1146,11 @@
       <c r="S12" s="9"/>
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
-    </row>
-    <row r="13" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V12" s="9"/>
+      <c r="W12" s="9"/>
+      <c r="X12" s="9"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -1101,8 +1172,11 @@
       <c r="S13" s="9"/>
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
-    </row>
-    <row r="14" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -1124,8 +1198,11 @@
       <c r="S14" s="9"/>
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
-    </row>
-    <row r="15" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V14" s="9"/>
+      <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -1147,8 +1224,11 @@
       <c r="S15" s="9"/>
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
-    </row>
-    <row r="16" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -1170,8 +1250,11 @@
       <c r="S16" s="9"/>
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
-    </row>
-    <row r="17" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V16" s="9"/>
+      <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -1193,8 +1276,11 @@
       <c r="S17" s="9"/>
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
-    </row>
-    <row r="18" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -1216,8 +1302,11 @@
       <c r="S18" s="9"/>
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
-    </row>
-    <row r="19" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -1239,8 +1328,11 @@
       <c r="S19" s="9"/>
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
-    </row>
-    <row r="20" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V19" s="9"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1262,8 +1354,11 @@
       <c r="S20" s="9"/>
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
-    </row>
-    <row r="21" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V20" s="9"/>
+      <c r="W20" s="9"/>
+      <c r="X20" s="9"/>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -1285,8 +1380,11 @@
       <c r="S21" s="9"/>
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
-    </row>
-    <row r="22" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V21" s="9"/>
+      <c r="W21" s="9"/>
+      <c r="X21" s="9"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -1308,8 +1406,11 @@
       <c r="S22" s="9"/>
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
-    </row>
-    <row r="23" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V22" s="9"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="9"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -1331,8 +1432,11 @@
       <c r="S23" s="9"/>
       <c r="T23" s="9"/>
       <c r="U23" s="9"/>
-    </row>
-    <row r="24" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V23" s="9"/>
+      <c r="W23" s="9"/>
+      <c r="X23" s="9"/>
+    </row>
+    <row r="24" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -1354,8 +1458,11 @@
       <c r="S24" s="9"/>
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
-    </row>
-    <row r="25" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V24" s="9"/>
+      <c r="W24" s="9"/>
+      <c r="X24" s="9"/>
+    </row>
+    <row r="25" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -1377,8 +1484,11 @@
       <c r="S25" s="9"/>
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
-    </row>
-    <row r="26" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V25" s="9"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
+    </row>
+    <row r="26" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -1400,8 +1510,11 @@
       <c r="S26" s="9"/>
       <c r="T26" s="9"/>
       <c r="U26" s="9"/>
-    </row>
-    <row r="27" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V26" s="9"/>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+    </row>
+    <row r="27" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -1423,8 +1536,11 @@
       <c r="S27" s="9"/>
       <c r="T27" s="9"/>
       <c r="U27" s="9"/>
-    </row>
-    <row r="28" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V27" s="9"/>
+      <c r="W27" s="9"/>
+      <c r="X27" s="9"/>
+    </row>
+    <row r="28" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -1446,8 +1562,11 @@
       <c r="S28" s="9"/>
       <c r="T28" s="9"/>
       <c r="U28" s="9"/>
-    </row>
-    <row r="29" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V28" s="9"/>
+      <c r="W28" s="9"/>
+      <c r="X28" s="9"/>
+    </row>
+    <row r="29" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -1469,8 +1588,11 @@
       <c r="S29" s="9"/>
       <c r="T29" s="9"/>
       <c r="U29" s="9"/>
-    </row>
-    <row r="30" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V29" s="9"/>
+      <c r="W29" s="9"/>
+      <c r="X29" s="9"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -1492,8 +1614,11 @@
       <c r="S30" s="9"/>
       <c r="T30" s="9"/>
       <c r="U30" s="9"/>
-    </row>
-    <row r="31" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V30" s="9"/>
+      <c r="W30" s="9"/>
+      <c r="X30" s="9"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -1515,8 +1640,11 @@
       <c r="S31" s="9"/>
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
-    </row>
-    <row r="32" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V31" s="9"/>
+      <c r="W31" s="9"/>
+      <c r="X31" s="9"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1538,8 +1666,11 @@
       <c r="S32" s="9"/>
       <c r="T32" s="9"/>
       <c r="U32" s="9"/>
-    </row>
-    <row r="33" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V32" s="9"/>
+      <c r="W32" s="9"/>
+      <c r="X32" s="9"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1561,8 +1692,11 @@
       <c r="S33" s="9"/>
       <c r="T33" s="9"/>
       <c r="U33" s="9"/>
-    </row>
-    <row r="34" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1584,8 +1718,11 @@
       <c r="S34" s="9"/>
       <c r="T34" s="9"/>
       <c r="U34" s="9"/>
-    </row>
-    <row r="35" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+    </row>
+    <row r="35" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1607,8 +1744,11 @@
       <c r="S35" s="9"/>
       <c r="T35" s="9"/>
       <c r="U35" s="9"/>
-    </row>
-    <row r="36" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+    </row>
+    <row r="36" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -1630,8 +1770,11 @@
       <c r="S36" s="9"/>
       <c r="T36" s="9"/>
       <c r="U36" s="9"/>
-    </row>
-    <row r="37" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+    </row>
+    <row r="37" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -1653,8 +1796,11 @@
       <c r="S37" s="9"/>
       <c r="T37" s="9"/>
       <c r="U37" s="9"/>
-    </row>
-    <row r="38" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V37" s="9"/>
+      <c r="W37" s="9"/>
+      <c r="X37" s="9"/>
+    </row>
+    <row r="38" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -1676,8 +1822,11 @@
       <c r="S38" s="9"/>
       <c r="T38" s="9"/>
       <c r="U38" s="9"/>
-    </row>
-    <row r="39" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V38" s="9"/>
+      <c r="W38" s="9"/>
+      <c r="X38" s="9"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -1699,8 +1848,11 @@
       <c r="S39" s="9"/>
       <c r="T39" s="9"/>
       <c r="U39" s="9"/>
-    </row>
-    <row r="40" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V39" s="9"/>
+      <c r="W39" s="9"/>
+      <c r="X39" s="9"/>
+    </row>
+    <row r="40" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
@@ -1722,8 +1874,11 @@
       <c r="S40" s="9"/>
       <c r="T40" s="9"/>
       <c r="U40" s="9"/>
-    </row>
-    <row r="41" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V40" s="9"/>
+      <c r="W40" s="9"/>
+      <c r="X40" s="9"/>
+    </row>
+    <row r="41" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -1745,8 +1900,11 @@
       <c r="S41" s="9"/>
       <c r="T41" s="9"/>
       <c r="U41" s="9"/>
-    </row>
-    <row r="42" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V41" s="9"/>
+      <c r="W41" s="9"/>
+      <c r="X41" s="9"/>
+    </row>
+    <row r="42" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" s="9"/>
       <c r="C42" s="9"/>
@@ -1768,8 +1926,11 @@
       <c r="S42" s="9"/>
       <c r="T42" s="9"/>
       <c r="U42" s="9"/>
-    </row>
-    <row r="43" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V42" s="9"/>
+      <c r="W42" s="9"/>
+      <c r="X42" s="9"/>
+    </row>
+    <row r="43" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -1791,8 +1952,11 @@
       <c r="S43" s="9"/>
       <c r="T43" s="9"/>
       <c r="U43" s="9"/>
-    </row>
-    <row r="44" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V43" s="9"/>
+      <c r="W43" s="9"/>
+      <c r="X43" s="9"/>
+    </row>
+    <row r="44" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -1814,8 +1978,11 @@
       <c r="S44" s="9"/>
       <c r="T44" s="9"/>
       <c r="U44" s="9"/>
-    </row>
-    <row r="45" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V44" s="9"/>
+      <c r="W44" s="9"/>
+      <c r="X44" s="9"/>
+    </row>
+    <row r="45" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
@@ -1837,8 +2004,11 @@
       <c r="S45" s="9"/>
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
-    </row>
-    <row r="46" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V45" s="9"/>
+      <c r="W45" s="9"/>
+      <c r="X45" s="9"/>
+    </row>
+    <row r="46" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -1860,8 +2030,11 @@
       <c r="S46" s="9"/>
       <c r="T46" s="9"/>
       <c r="U46" s="9"/>
-    </row>
-    <row r="47" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V46" s="9"/>
+      <c r="W46" s="9"/>
+      <c r="X46" s="9"/>
+    </row>
+    <row r="47" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
       <c r="B47" s="9"/>
       <c r="C47" s="9"/>
@@ -1883,8 +2056,11 @@
       <c r="S47" s="9"/>
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
-    </row>
-    <row r="48" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V47" s="9"/>
+      <c r="W47" s="9"/>
+      <c r="X47" s="9"/>
+    </row>
+    <row r="48" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
       <c r="B48" s="9"/>
       <c r="C48" s="9"/>
@@ -1906,8 +2082,11 @@
       <c r="S48" s="9"/>
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
-    </row>
-    <row r="49" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V48" s="9"/>
+      <c r="W48" s="9"/>
+      <c r="X48" s="9"/>
+    </row>
+    <row r="49" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
       <c r="B49" s="9"/>
       <c r="C49" s="9"/>
@@ -1929,8 +2108,11 @@
       <c r="S49" s="9"/>
       <c r="T49" s="9"/>
       <c r="U49" s="9"/>
-    </row>
-    <row r="50" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V49" s="9"/>
+      <c r="W49" s="9"/>
+      <c r="X49" s="9"/>
+    </row>
+    <row r="50" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
@@ -1952,8 +2134,11 @@
       <c r="S50" s="9"/>
       <c r="T50" s="9"/>
       <c r="U50" s="9"/>
-    </row>
-    <row r="51" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V50" s="9"/>
+      <c r="W50" s="9"/>
+      <c r="X50" s="9"/>
+    </row>
+    <row r="51" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -1975,8 +2160,11 @@
       <c r="S51" s="9"/>
       <c r="T51" s="9"/>
       <c r="U51" s="9"/>
-    </row>
-    <row r="52" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V51" s="9"/>
+      <c r="W51" s="9"/>
+      <c r="X51" s="9"/>
+    </row>
+    <row r="52" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
       <c r="C52" s="9"/>
@@ -1998,8 +2186,11 @@
       <c r="S52" s="9"/>
       <c r="T52" s="9"/>
       <c r="U52" s="9"/>
-    </row>
-    <row r="53" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V52" s="9"/>
+      <c r="W52" s="9"/>
+      <c r="X52" s="9"/>
+    </row>
+    <row r="53" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
       <c r="B53" s="9"/>
       <c r="C53" s="9"/>
@@ -2021,8 +2212,11 @@
       <c r="S53" s="9"/>
       <c r="T53" s="9"/>
       <c r="U53" s="9"/>
-    </row>
-    <row r="54" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V53" s="9"/>
+      <c r="W53" s="9"/>
+      <c r="X53" s="9"/>
+    </row>
+    <row r="54" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
       <c r="B54" s="9"/>
       <c r="C54" s="9"/>
@@ -2044,8 +2238,11 @@
       <c r="S54" s="9"/>
       <c r="T54" s="9"/>
       <c r="U54" s="9"/>
-    </row>
-    <row r="55" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V54" s="9"/>
+      <c r="W54" s="9"/>
+      <c r="X54" s="9"/>
+    </row>
+    <row r="55" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
@@ -2067,8 +2264,11 @@
       <c r="S55" s="9"/>
       <c r="T55" s="9"/>
       <c r="U55" s="9"/>
-    </row>
-    <row r="56" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V55" s="9"/>
+      <c r="W55" s="9"/>
+      <c r="X55" s="9"/>
+    </row>
+    <row r="56" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
       <c r="B56" s="9"/>
       <c r="C56" s="9"/>
@@ -2090,8 +2290,11 @@
       <c r="S56" s="9"/>
       <c r="T56" s="9"/>
       <c r="U56" s="9"/>
-    </row>
-    <row r="57" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V56" s="9"/>
+      <c r="W56" s="9"/>
+      <c r="X56" s="9"/>
+    </row>
+    <row r="57" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
       <c r="B57" s="9"/>
       <c r="C57" s="9"/>
@@ -2113,8 +2316,11 @@
       <c r="S57" s="9"/>
       <c r="T57" s="9"/>
       <c r="U57" s="9"/>
-    </row>
-    <row r="58" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V57" s="9"/>
+      <c r="W57" s="9"/>
+      <c r="X57" s="9"/>
+    </row>
+    <row r="58" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="B58" s="9"/>
       <c r="C58" s="9"/>
@@ -2136,8 +2342,11 @@
       <c r="S58" s="9"/>
       <c r="T58" s="9"/>
       <c r="U58" s="9"/>
-    </row>
-    <row r="59" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V58" s="9"/>
+      <c r="W58" s="9"/>
+      <c r="X58" s="9"/>
+    </row>
+    <row r="59" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A59" s="9"/>
       <c r="B59" s="9"/>
       <c r="C59" s="9"/>
@@ -2159,8 +2368,11 @@
       <c r="S59" s="9"/>
       <c r="T59" s="9"/>
       <c r="U59" s="9"/>
-    </row>
-    <row r="60" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V59" s="9"/>
+      <c r="W59" s="9"/>
+      <c r="X59" s="9"/>
+    </row>
+    <row r="60" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
       <c r="B60" s="9"/>
       <c r="C60" s="9"/>
@@ -2182,8 +2394,11 @@
       <c r="S60" s="9"/>
       <c r="T60" s="9"/>
       <c r="U60" s="9"/>
-    </row>
-    <row r="61" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V60" s="9"/>
+      <c r="W60" s="9"/>
+      <c r="X60" s="9"/>
+    </row>
+    <row r="61" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -2205,8 +2420,11 @@
       <c r="S61" s="9"/>
       <c r="T61" s="9"/>
       <c r="U61" s="9"/>
-    </row>
-    <row r="62" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V61" s="9"/>
+      <c r="W61" s="9"/>
+      <c r="X61" s="9"/>
+    </row>
+    <row r="62" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A62" s="9"/>
       <c r="B62" s="9"/>
       <c r="C62" s="9"/>
@@ -2228,8 +2446,11 @@
       <c r="S62" s="9"/>
       <c r="T62" s="9"/>
       <c r="U62" s="9"/>
-    </row>
-    <row r="63" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V62" s="9"/>
+      <c r="W62" s="9"/>
+      <c r="X62" s="9"/>
+    </row>
+    <row r="63" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -2251,8 +2472,11 @@
       <c r="S63" s="9"/>
       <c r="T63" s="9"/>
       <c r="U63" s="9"/>
-    </row>
-    <row r="64" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V63" s="9"/>
+      <c r="W63" s="9"/>
+      <c r="X63" s="9"/>
+    </row>
+    <row r="64" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A64" s="9"/>
       <c r="B64" s="9"/>
       <c r="C64" s="9"/>
@@ -2274,8 +2498,11 @@
       <c r="S64" s="9"/>
       <c r="T64" s="9"/>
       <c r="U64" s="9"/>
-    </row>
-    <row r="65" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V64" s="9"/>
+      <c r="W64" s="9"/>
+      <c r="X64" s="9"/>
+    </row>
+    <row r="65" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
@@ -2297,8 +2524,11 @@
       <c r="S65" s="9"/>
       <c r="T65" s="9"/>
       <c r="U65" s="9"/>
-    </row>
-    <row r="66" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V65" s="9"/>
+      <c r="W65" s="9"/>
+      <c r="X65" s="9"/>
+    </row>
+    <row r="66" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
@@ -2320,8 +2550,11 @@
       <c r="S66" s="9"/>
       <c r="T66" s="9"/>
       <c r="U66" s="9"/>
-    </row>
-    <row r="67" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V66" s="9"/>
+      <c r="W66" s="9"/>
+      <c r="X66" s="9"/>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A67" s="9"/>
       <c r="B67" s="9"/>
       <c r="C67" s="9"/>
@@ -2343,8 +2576,11 @@
       <c r="S67" s="9"/>
       <c r="T67" s="9"/>
       <c r="U67" s="9"/>
-    </row>
-    <row r="68" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V67" s="9"/>
+      <c r="W67" s="9"/>
+      <c r="X67" s="9"/>
+    </row>
+    <row r="68" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A68" s="9"/>
       <c r="B68" s="9"/>
       <c r="C68" s="9"/>
@@ -2366,8 +2602,11 @@
       <c r="S68" s="9"/>
       <c r="T68" s="9"/>
       <c r="U68" s="9"/>
-    </row>
-    <row r="69" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V68" s="9"/>
+      <c r="W68" s="9"/>
+      <c r="X68" s="9"/>
+    </row>
+    <row r="69" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A69" s="9"/>
       <c r="B69" s="9"/>
       <c r="C69" s="9"/>
@@ -2389,8 +2628,11 @@
       <c r="S69" s="9"/>
       <c r="T69" s="9"/>
       <c r="U69" s="9"/>
-    </row>
-    <row r="70" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V69" s="9"/>
+      <c r="W69" s="9"/>
+      <c r="X69" s="9"/>
+    </row>
+    <row r="70" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -2412,8 +2654,11 @@
       <c r="S70" s="9"/>
       <c r="T70" s="9"/>
       <c r="U70" s="9"/>
-    </row>
-    <row r="71" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V70" s="9"/>
+      <c r="W70" s="9"/>
+      <c r="X70" s="9"/>
+    </row>
+    <row r="71" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A71" s="9"/>
       <c r="B71" s="9"/>
       <c r="C71" s="9"/>
@@ -2435,8 +2680,11 @@
       <c r="S71" s="9"/>
       <c r="T71" s="9"/>
       <c r="U71" s="9"/>
-    </row>
-    <row r="72" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V71" s="9"/>
+      <c r="W71" s="9"/>
+      <c r="X71" s="9"/>
+    </row>
+    <row r="72" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A72" s="9"/>
       <c r="B72" s="9"/>
       <c r="C72" s="9"/>
@@ -2458,8 +2706,11 @@
       <c r="S72" s="9"/>
       <c r="T72" s="9"/>
       <c r="U72" s="9"/>
-    </row>
-    <row r="73" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V72" s="9"/>
+      <c r="W72" s="9"/>
+      <c r="X72" s="9"/>
+    </row>
+    <row r="73" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A73" s="9"/>
       <c r="B73" s="9"/>
       <c r="C73" s="9"/>
@@ -2481,8 +2732,11 @@
       <c r="S73" s="9"/>
       <c r="T73" s="9"/>
       <c r="U73" s="9"/>
-    </row>
-    <row r="74" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V73" s="9"/>
+      <c r="W73" s="9"/>
+      <c r="X73" s="9"/>
+    </row>
+    <row r="74" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A74" s="9"/>
       <c r="B74" s="9"/>
       <c r="C74" s="9"/>
@@ -2504,8 +2758,11 @@
       <c r="S74" s="9"/>
       <c r="T74" s="9"/>
       <c r="U74" s="9"/>
-    </row>
-    <row r="75" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V74" s="9"/>
+      <c r="W74" s="9"/>
+      <c r="X74" s="9"/>
+    </row>
+    <row r="75" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A75" s="9"/>
       <c r="B75" s="9"/>
       <c r="C75" s="9"/>
@@ -2527,8 +2784,11 @@
       <c r="S75" s="9"/>
       <c r="T75" s="9"/>
       <c r="U75" s="9"/>
-    </row>
-    <row r="76" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V75" s="9"/>
+      <c r="W75" s="9"/>
+      <c r="X75" s="9"/>
+    </row>
+    <row r="76" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A76" s="9"/>
       <c r="B76" s="9"/>
       <c r="C76" s="9"/>
@@ -2550,8 +2810,11 @@
       <c r="S76" s="9"/>
       <c r="T76" s="9"/>
       <c r="U76" s="9"/>
-    </row>
-    <row r="77" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V76" s="9"/>
+      <c r="W76" s="9"/>
+      <c r="X76" s="9"/>
+    </row>
+    <row r="77" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A77" s="9"/>
       <c r="B77" s="9"/>
       <c r="C77" s="9"/>
@@ -2573,8 +2836,11 @@
       <c r="S77" s="9"/>
       <c r="T77" s="9"/>
       <c r="U77" s="9"/>
-    </row>
-    <row r="78" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V77" s="9"/>
+      <c r="W77" s="9"/>
+      <c r="X77" s="9"/>
+    </row>
+    <row r="78" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A78" s="9"/>
       <c r="B78" s="9"/>
       <c r="C78" s="9"/>
@@ -2596,8 +2862,11 @@
       <c r="S78" s="9"/>
       <c r="T78" s="9"/>
       <c r="U78" s="9"/>
-    </row>
-    <row r="79" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V78" s="9"/>
+      <c r="W78" s="9"/>
+      <c r="X78" s="9"/>
+    </row>
+    <row r="79" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
       <c r="B79" s="9"/>
       <c r="C79" s="9"/>
@@ -2619,8 +2888,11 @@
       <c r="S79" s="9"/>
       <c r="T79" s="9"/>
       <c r="U79" s="9"/>
-    </row>
-    <row r="80" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V79" s="9"/>
+      <c r="W79" s="9"/>
+      <c r="X79" s="9"/>
+    </row>
+    <row r="80" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
       <c r="B80" s="9"/>
       <c r="C80" s="9"/>
@@ -2642,8 +2914,11 @@
       <c r="S80" s="9"/>
       <c r="T80" s="9"/>
       <c r="U80" s="9"/>
-    </row>
-    <row r="81" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V80" s="9"/>
+      <c r="W80" s="9"/>
+      <c r="X80" s="9"/>
+    </row>
+    <row r="81" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A81" s="9"/>
       <c r="B81" s="9"/>
       <c r="C81" s="9"/>
@@ -2665,8 +2940,11 @@
       <c r="S81" s="9"/>
       <c r="T81" s="9"/>
       <c r="U81" s="9"/>
-    </row>
-    <row r="82" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V81" s="9"/>
+      <c r="W81" s="9"/>
+      <c r="X81" s="9"/>
+    </row>
+    <row r="82" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A82" s="9"/>
       <c r="B82" s="9"/>
       <c r="C82" s="9"/>
@@ -2688,8 +2966,11 @@
       <c r="S82" s="9"/>
       <c r="T82" s="9"/>
       <c r="U82" s="9"/>
-    </row>
-    <row r="83" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V82" s="9"/>
+      <c r="W82" s="9"/>
+      <c r="X82" s="9"/>
+    </row>
+    <row r="83" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
       <c r="B83" s="9"/>
       <c r="C83" s="9"/>
@@ -2711,8 +2992,11 @@
       <c r="S83" s="9"/>
       <c r="T83" s="9"/>
       <c r="U83" s="9"/>
-    </row>
-    <row r="84" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V83" s="9"/>
+      <c r="W83" s="9"/>
+      <c r="X83" s="9"/>
+    </row>
+    <row r="84" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A84" s="9"/>
       <c r="B84" s="9"/>
       <c r="C84" s="9"/>
@@ -2734,8 +3018,11 @@
       <c r="S84" s="9"/>
       <c r="T84" s="9"/>
       <c r="U84" s="9"/>
-    </row>
-    <row r="85" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V84" s="9"/>
+      <c r="W84" s="9"/>
+      <c r="X84" s="9"/>
+    </row>
+    <row r="85" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
       <c r="B85" s="9"/>
       <c r="C85" s="9"/>
@@ -2757,8 +3044,11 @@
       <c r="S85" s="9"/>
       <c r="T85" s="9"/>
       <c r="U85" s="9"/>
-    </row>
-    <row r="86" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V85" s="9"/>
+      <c r="W85" s="9"/>
+      <c r="X85" s="9"/>
+    </row>
+    <row r="86" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
       <c r="B86" s="9"/>
       <c r="C86" s="9"/>
@@ -2780,8 +3070,11 @@
       <c r="S86" s="9"/>
       <c r="T86" s="9"/>
       <c r="U86" s="9"/>
-    </row>
-    <row r="87" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V86" s="9"/>
+      <c r="W86" s="9"/>
+      <c r="X86" s="9"/>
+    </row>
+    <row r="87" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A87" s="9"/>
       <c r="B87" s="9"/>
       <c r="C87" s="9"/>
@@ -2803,8 +3096,11 @@
       <c r="S87" s="9"/>
       <c r="T87" s="9"/>
       <c r="U87" s="9"/>
-    </row>
-    <row r="88" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V87" s="9"/>
+      <c r="W87" s="9"/>
+      <c r="X87" s="9"/>
+    </row>
+    <row r="88" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
       <c r="B88" s="9"/>
       <c r="C88" s="9"/>
@@ -2826,8 +3122,11 @@
       <c r="S88" s="9"/>
       <c r="T88" s="9"/>
       <c r="U88" s="9"/>
-    </row>
-    <row r="89" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V88" s="9"/>
+      <c r="W88" s="9"/>
+      <c r="X88" s="9"/>
+    </row>
+    <row r="89" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
       <c r="B89" s="9"/>
       <c r="C89" s="9"/>
@@ -2849,8 +3148,11 @@
       <c r="S89" s="9"/>
       <c r="T89" s="9"/>
       <c r="U89" s="9"/>
-    </row>
-    <row r="90" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V89" s="9"/>
+      <c r="W89" s="9"/>
+      <c r="X89" s="9"/>
+    </row>
+    <row r="90" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
       <c r="B90" s="9"/>
       <c r="C90" s="9"/>
@@ -2872,8 +3174,11 @@
       <c r="S90" s="9"/>
       <c r="T90" s="9"/>
       <c r="U90" s="9"/>
-    </row>
-    <row r="91" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V90" s="9"/>
+      <c r="W90" s="9"/>
+      <c r="X90" s="9"/>
+    </row>
+    <row r="91" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
       <c r="B91" s="9"/>
       <c r="C91" s="9"/>
@@ -2895,8 +3200,11 @@
       <c r="S91" s="9"/>
       <c r="T91" s="9"/>
       <c r="U91" s="9"/>
-    </row>
-    <row r="92" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V91" s="9"/>
+      <c r="W91" s="9"/>
+      <c r="X91" s="9"/>
+    </row>
+    <row r="92" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
       <c r="B92" s="9"/>
       <c r="C92" s="9"/>
@@ -2918,8 +3226,11 @@
       <c r="S92" s="9"/>
       <c r="T92" s="9"/>
       <c r="U92" s="9"/>
-    </row>
-    <row r="93" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V92" s="9"/>
+      <c r="W92" s="9"/>
+      <c r="X92" s="9"/>
+    </row>
+    <row r="93" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A93" s="9"/>
       <c r="B93" s="9"/>
       <c r="C93" s="9"/>
@@ -2941,8 +3252,11 @@
       <c r="S93" s="9"/>
       <c r="T93" s="9"/>
       <c r="U93" s="9"/>
-    </row>
-    <row r="94" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V93" s="9"/>
+      <c r="W93" s="9"/>
+      <c r="X93" s="9"/>
+    </row>
+    <row r="94" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A94" s="9"/>
       <c r="B94" s="9"/>
       <c r="C94" s="9"/>
@@ -2964,8 +3278,11 @@
       <c r="S94" s="9"/>
       <c r="T94" s="9"/>
       <c r="U94" s="9"/>
-    </row>
-    <row r="95" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V94" s="9"/>
+      <c r="W94" s="9"/>
+      <c r="X94" s="9"/>
+    </row>
+    <row r="95" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
       <c r="B95" s="9"/>
       <c r="C95" s="9"/>
@@ -2987,8 +3304,11 @@
       <c r="S95" s="9"/>
       <c r="T95" s="9"/>
       <c r="U95" s="9"/>
-    </row>
-    <row r="96" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V95" s="9"/>
+      <c r="W95" s="9"/>
+      <c r="X95" s="9"/>
+    </row>
+    <row r="96" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A96" s="9"/>
       <c r="B96" s="9"/>
       <c r="C96" s="9"/>
@@ -3010,8 +3330,11 @@
       <c r="S96" s="9"/>
       <c r="T96" s="9"/>
       <c r="U96" s="9"/>
-    </row>
-    <row r="97" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V96" s="9"/>
+      <c r="W96" s="9"/>
+      <c r="X96" s="9"/>
+    </row>
+    <row r="97" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A97" s="9"/>
       <c r="B97" s="9"/>
       <c r="C97" s="9"/>
@@ -3033,8 +3356,11 @@
       <c r="S97" s="9"/>
       <c r="T97" s="9"/>
       <c r="U97" s="9"/>
-    </row>
-    <row r="98" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V97" s="9"/>
+      <c r="W97" s="9"/>
+      <c r="X97" s="9"/>
+    </row>
+    <row r="98" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
       <c r="B98" s="9"/>
       <c r="C98" s="9"/>
@@ -3056,8 +3382,11 @@
       <c r="S98" s="9"/>
       <c r="T98" s="9"/>
       <c r="U98" s="9"/>
-    </row>
-    <row r="99" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V98" s="9"/>
+      <c r="W98" s="9"/>
+      <c r="X98" s="9"/>
+    </row>
+    <row r="99" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A99" s="9"/>
       <c r="B99" s="9"/>
       <c r="C99" s="9"/>
@@ -3079,8 +3408,11 @@
       <c r="S99" s="9"/>
       <c r="T99" s="9"/>
       <c r="U99" s="9"/>
-    </row>
-    <row r="100" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V99" s="9"/>
+      <c r="W99" s="9"/>
+      <c r="X99" s="9"/>
+    </row>
+    <row r="100" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
       <c r="B100" s="9"/>
       <c r="C100" s="9"/>
@@ -3102,8 +3434,11 @@
       <c r="S100" s="9"/>
       <c r="T100" s="9"/>
       <c r="U100" s="9"/>
-    </row>
-    <row r="101" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V100" s="9"/>
+      <c r="W100" s="9"/>
+      <c r="X100" s="9"/>
+    </row>
+    <row r="101" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A101" s="9"/>
       <c r="B101" s="9"/>
       <c r="C101" s="9"/>
@@ -3125,8 +3460,11 @@
       <c r="S101" s="9"/>
       <c r="T101" s="9"/>
       <c r="U101" s="9"/>
-    </row>
-    <row r="102" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V101" s="9"/>
+      <c r="W101" s="9"/>
+      <c r="X101" s="9"/>
+    </row>
+    <row r="102" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A102" s="9"/>
       <c r="B102" s="9"/>
       <c r="C102" s="9"/>
@@ -3148,8 +3486,11 @@
       <c r="S102" s="9"/>
       <c r="T102" s="9"/>
       <c r="U102" s="9"/>
-    </row>
-    <row r="103" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="V102" s="9"/>
+      <c r="W102" s="9"/>
+      <c r="X102" s="9"/>
+    </row>
+    <row r="103" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A103" s="9"/>
       <c r="B103" s="9"/>
       <c r="C103" s="9"/>
@@ -3171,9 +3512,12 @@
       <c r="S103" s="9"/>
       <c r="T103" s="9"/>
       <c r="U103" s="9"/>
+      <c r="V103" s="9"/>
+      <c r="W103" s="9"/>
+      <c r="X103" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>